<commit_message>
Stakeholder Matrix gets an Email column; workshop-summary uses it for recipients
- templates-source/discovery-setup/stakeholder-matrix.xlsx: Email after
  Organization; dropdowns and widths shifted; templates.json rebuilt
- workshop-summary: recipients from the calendar invite, else from the
  Stakeholder Matrix by exact name; the gate shows where each email came from
- New eval case workshop-summary-emails-from-matrix (passes, 1 run)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JEt3XhtRwUHbEHNFmAvqPW
</commit_message>
<xml_diff>
--- a/templates-source/discovery-setup/stakeholder-matrix.xlsx
+++ b/templates-source/discovery-setup/stakeholder-matrix.xlsx
@@ -422,17 +422,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -453,25 +454,30 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Influence</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Interest</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Attitude</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>How to engage</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -479,13 +485,13 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"High,Medium,Low"</formula1>
-    </dataValidation>
     <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"High,Medium,Low"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Supporter,Neutral,Skeptic"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>